<commit_message>
Refresh cached Box snapshot before importing metadata
</commit_message>
<xml_diff>
--- a/data/inputs/Metrics captured by database_ACTIVE.xlsx
+++ b/data/inputs/Metrics captured by database_ACTIVE.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29922"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30110"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="1672" documentId="13_ncr:1_{D5D2EC57-4ADD-414D-A620-51AA4D9E28A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AB5A776-8BDB-4F75-9033-324365B013A4}"/>
+  <xr:revisionPtr revIDLastSave="1719" documentId="13_ncr:1_{D5D2EC57-4ADD-414D-A620-51AA4D9E28A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{241FDDC5-2F7D-41A3-B8EE-36A3BC587DB2}"/>
   <bookViews>
-    <workbookView xWindow="72960" yWindow="0" windowWidth="38400" windowHeight="21600" firstSheet="3" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="72960" yWindow="0" windowWidth="38400" windowHeight="21600" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current state of SHAPE" sheetId="4" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="373">
   <si>
     <t>Health Assessment Domain</t>
   </si>
@@ -255,7 +255,7 @@
     <t>Food insecurity</t>
   </si>
   <si>
-    <t>ACS, BRFSS, CIF, NHIS, HINTS</t>
+    <t>BRFSS, CIF, NHIS, HINTS</t>
   </si>
   <si>
     <t>DOH</t>
@@ -291,7 +291,7 @@
     <t>EDW (no substantial data available)</t>
   </si>
   <si>
-    <t>Persons below 150% of poverty, 2017-2021</t>
+    <t>Persons below 150% of poverty</t>
   </si>
   <si>
     <t>ACS, SVI</t>
@@ -434,6 +434,9 @@
     <t>Census tract</t>
   </si>
   <si>
+    <t>Persons below 150% of poverty, 2017-2021</t>
+  </si>
+  <si>
     <t xml:space="preserve">wellbeing/mental health/emotional wellbeing </t>
   </si>
   <si>
@@ -452,7 +455,7 @@
     <t>All variables by Race/ethnicity and sex: All sites, Young adult, Alcohol associated, Bladder, Brain, Cervix, Cervix 21-65, Cervix early stage, Cervix late stage, Colon/rectum, Colon/rectum 45-75, Colon/rectum early stage, Colon/rectum late stage, Uterus, Esophagus, Female breast, Female breast 40-74, Female breast early stage, Female breast late stage, HPV associated, Head and neck, Kidney renal pelvis, Leukemia, Liver IBD, Lung bronchus, Lung bronchus 50-80, Lung bronchus early stage, Lung bronchus late stage, Melanoma, Non-Hodgkin lymphoma, Obesity associated, Oral Cavity Pharynx, Ovary, Pancreas, Pediatric, Prostate, Stomach, Thyroid, Tobacco associated</t>
   </si>
   <si>
-    <t>5-year average age-adjusted rates over 2017-2021</t>
+    <t>5-year average age-adjusted rates over 2018-2022</t>
   </si>
   <si>
     <t>This data comes from a direct connection into their database, but here is their website: https://www.cdc.gov/united-states-cancer-statistics/index.html</t>
@@ -461,7 +464,7 @@
     <t>All variables by Race/ethnicity and sex: All sites, Bladder, Brain, Cervix, Colon/rectum, Uterus, Esophagus, Female breast, Kidney renal pelvis, Leukemia, Liver IBD, Lung bronchus, Melanoma, Non-Hodgkin lymphoma, Oral Cavity Pharynx, Ovary, Pancreas, Prostate, Stomach, Thyroid</t>
   </si>
   <si>
-    <t>5-year average age-adjusted rates over 2018-2022</t>
+    <t>5-year average age-adjusted rates over 2019-2023</t>
   </si>
   <si>
     <t>https://statecancerprofiles.cancer.gov/index.html</t>
@@ -506,7 +509,7 @@
     <t>I am not sure if these variables are exactly what you're looking for, but I thought some of them might apply: Uninsured children, Uninsured black, Uninsured hispanic, Living below poverty black, Living below poverty hispanic, Insurance coverage, Household income, Annual unemployment, Below poverty, Uninsured, Rent burden over 40% of income</t>
   </si>
   <si>
-    <t>2018-2022</t>
+    <t>2020-2024</t>
   </si>
   <si>
     <t>https://data.census.gov/</t>
@@ -521,7 +524,7 @@
     <t>Food deserts, Food insecure</t>
   </si>
   <si>
-    <t>Deserts: 2015, Insecure: 2022</t>
+    <t>Deserts: 2019, Insecure: 2022</t>
   </si>
   <si>
     <t>Deserts: https://www.ers.usda.gov/data-products/food-access-research-atlas/, Insecure: https://www.cdc.gov/places/</t>
@@ -530,7 +533,7 @@
     <t>Housing insecure, Multi-unit structures, Mobile homes, Owner occupied housing, Crowded housing, Lack complete plumbing, Median home value, Median monthly mortgage, Median gross rent, No home broadband, Rent burden 40% of income</t>
   </si>
   <si>
-    <t>Insecure: 2022, the other variables: 2018-2022</t>
+    <t>Insecure: 2022, the other variables: 2020-2024</t>
   </si>
   <si>
     <t>Insecure: https://www.cdc.gov/places/, the other variables: https://data.census.gov/</t>
@@ -545,7 +548,7 @@
     <t>Have to verify some of the definitions, but this is about speeds I believe: pctBB100010, pctBB10020, pct5G71, pct5G353, No home broadband</t>
   </si>
   <si>
-    <t>First four: Dec 2023, Last one: 2018-2022</t>
+    <t>First four: Dec 2024, Last one: 2020-2024</t>
   </si>
   <si>
     <t>First four: https://broadbandmap.fcc.gov/home, Last one: https://data.census.gov/</t>
@@ -557,6 +560,9 @@
     <t>Have you ever had a mammogram?; Women respondents aged 40+ who have had a mammogram in the past two years; Women respondents aged 50-74 who have had a mammogram in the past two years; How long has it been since you had your last mammogram?</t>
   </si>
   <si>
+    <t>2022, 2024</t>
+  </si>
+  <si>
     <t>https://www.cdc.gov/brfss/annual_data/annual_data.htm</t>
   </si>
   <si>
@@ -590,7 +596,7 @@
     <t>Have you smoked at least 100 cigarettes in your entire life?[Note5 packs = 100 cigarettes]; Four-level smoker statusEveryday smoker, Someday smoker, Former smoker, Non-smoker; Adults who are current smokers</t>
   </si>
   <si>
-    <t>2022, 2023</t>
+    <t>2022, 2023, 2024</t>
   </si>
   <si>
     <t>Was there a time in the past 12 months when you needed to see a doctor but could not because you could not afford it?</t>
@@ -611,9 +617,6 @@
     <t>Now thinking about your mental health, which includes stress, depression, and problems with emotions, for how many days during the past 30 days was your mental health not good?</t>
   </si>
   <si>
-    <t>I have only gotten 2022 and 2023 data. If we want to observe trends over time, I can get more years.</t>
-  </si>
-  <si>
     <t>Stable measures weren't produced</t>
   </si>
   <si>
@@ -953,15 +956,12 @@
     <t>Is this person CURRENTLY covered by any of the following types of health insurance or health coverage plans? </t>
   </si>
   <si>
-    <t>2022 (5 year cycle)</t>
+    <t>2019-2023, 2020-2024 (5 year cycles)</t>
   </si>
   <si>
     <t>https://usa.ipums.org/usa-action/source_documents/enum_form_ACS(2022)_tag.xml</t>
   </si>
   <si>
-    <t> IN THE PAST 12 MONTHS, did you or any member of this household receive benefits from the Food Stamp Program or SNAP (the Supplemental Nutrition Assistance Program)? Do NOT include WIC, the School Lunch Program, or assistance from food banks.</t>
-  </si>
-  <si>
     <t>What was this person's total income during the PAST 12 MONTHS</t>
   </si>
   <si>
@@ -974,6 +974,9 @@
     <t>Can you or any member of this household both make and receive phone calls when at this house, apartment, or mobile home? Include calls using cell phones, land lines, or other phone devices..</t>
   </si>
   <si>
+    <t>2018-2022 (5 year cycle)</t>
+  </si>
+  <si>
     <t>At this house, apartment, or mobile home - do you or any member of this household own or use any of the following types of computers? Desktop or laptop; smartphone; tablet or other portable wireless computer; some other type of computer</t>
   </si>
   <si>
@@ -981,9 +984,6 @@
   </si>
   <si>
     <t>Good days, Moderate days, Unhealthy for sensitive groups days, Unhealthy days, Very unhealthy days, Hazardous days</t>
-  </si>
-  <si>
-    <t>1980-2024, but I only got the 2023 data (need to update)</t>
   </si>
   <si>
     <t>https://aqs.epa.gov/aqsweb/airdata/download_files.html</t>
@@ -2003,7 +2003,7 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="200">
+  <cellXfs count="207">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2553,6 +2553,27 @@
     <xf numFmtId="0" fontId="24" fillId="22" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
@@ -3397,7 +3418,7 @@
         <v>74</v>
       </c>
       <c r="C37" s="80" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="D37" s="46" t="s">
         <v>75</v>
@@ -3459,7 +3480,7 @@
         <v>83</v>
       </c>
       <c r="C41" s="84" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="D41" s="83" t="s">
         <v>84</v>
@@ -3643,7 +3664,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79CF1CD7-894F-4366-BBDA-3E50090B14D9}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="37.109375" bestFit="1" customWidth="1"/>
@@ -3657,13 +3678,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3674,18 +3695,18 @@
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
     </row>
-    <row r="3" spans="1:4" ht="16.5">
+    <row r="3" spans="1:4" ht="51.75" customHeight="1">
       <c r="A3" s="57" t="s">
         <v>45</v>
       </c>
       <c r="B3" s="130" t="s">
-        <v>297</v>
-      </c>
-      <c r="C3" s="119" t="s">
         <v>298</v>
       </c>
+      <c r="C3" s="194" t="s">
+        <v>299</v>
+      </c>
       <c r="D3" s="128" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -3697,115 +3718,100 @@
       <c r="D4" s="16"/>
     </row>
     <row r="5" spans="1:4" ht="48.75">
-      <c r="A5" s="76" t="s">
-        <v>66</v>
-      </c>
-      <c r="B5" s="131" t="s">
+      <c r="A5" s="79" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="126" t="s">
+        <v>301</v>
+      </c>
+      <c r="C5" s="131" t="s">
+        <v>299</v>
+      </c>
+      <c r="D5" s="131" t="s">
         <v>300</v>
       </c>
-      <c r="C5" s="131" t="s">
-        <v>298</v>
-      </c>
-      <c r="D5" s="131" t="s">
+    </row>
+    <row r="6" spans="1:4" ht="48.75">
+      <c r="A6" s="79" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="126" t="s">
+        <v>302</v>
+      </c>
+      <c r="C6" s="131" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="32.25">
-      <c r="A6" s="79" t="s">
-        <v>76</v>
-      </c>
-      <c r="B6" s="126" t="s">
-        <v>301</v>
-      </c>
-      <c r="C6" s="131" t="s">
-        <v>298</v>
-      </c>
       <c r="D6" s="131" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="16.5">
-      <c r="A7" s="79" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="126" t="s">
-        <v>302</v>
-      </c>
-      <c r="C7" s="131" t="s">
-        <v>298</v>
-      </c>
-      <c r="D7" s="131" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="28" t="s">
+    <row r="7" spans="1:4">
+      <c r="A7" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-    </row>
-    <row r="9" spans="1:4" ht="28.5">
-      <c r="A9" s="85" t="s">
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+    </row>
+    <row r="8" spans="1:4" ht="28.5">
+      <c r="A8" s="85" t="s">
         <v>88</v>
       </c>
+      <c r="B8" s="123" t="s">
+        <v>304</v>
+      </c>
+      <c r="C8" s="112" t="s">
+        <v>305</v>
+      </c>
+      <c r="D8" s="129" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="42.75">
+      <c r="A9" s="85"/>
       <c r="B9" s="123" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C9" s="112" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="D9" s="129" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="42.75">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16.5">
       <c r="A10" s="85"/>
       <c r="B10" s="123" t="s">
+        <v>245</v>
+      </c>
+      <c r="C10" s="112" t="s">
         <v>305</v>
       </c>
-      <c r="C10" s="112" t="s">
-        <v>298</v>
-      </c>
       <c r="D10" s="129" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="16.5">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="57">
       <c r="A11" s="85"/>
       <c r="B11" s="123" t="s">
-        <v>244</v>
+        <v>307</v>
       </c>
       <c r="C11" s="112" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="D11" s="129" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="57">
-      <c r="A12" s="85"/>
-      <c r="B12" s="123" t="s">
-        <v>306</v>
-      </c>
-      <c r="C12" s="112" t="s">
-        <v>298</v>
-      </c>
-      <c r="D12" s="129" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" xr:uid="{33DDCCAA-92C9-4F7E-882F-165AAD570669}"/>
-    <hyperlink ref="D5" r:id="rId2" xr:uid="{4BD13D57-27BF-4B32-B390-E02C3D8888BE}"/>
-    <hyperlink ref="D6" r:id="rId3" xr:uid="{903E4187-89B5-494B-A114-19A08F53DFF6}"/>
-    <hyperlink ref="D7" r:id="rId4" xr:uid="{C20B532B-CF38-45ED-A9A6-B0314F17708B}"/>
-    <hyperlink ref="D9" r:id="rId5" xr:uid="{6C0887D4-947C-4463-A546-6AB836B0B3D8}"/>
-    <hyperlink ref="D10" r:id="rId6" xr:uid="{F0533DB3-A661-4182-888A-949669537D09}"/>
-    <hyperlink ref="D11" r:id="rId7" xr:uid="{3C31B3A0-29AB-41BE-B877-46BE0AC5D6D5}"/>
-    <hyperlink ref="D12" r:id="rId8" xr:uid="{C0DAFC63-62EC-41DB-8DCD-5B75D22A1A2B}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{903E4187-89B5-494B-A114-19A08F53DFF6}"/>
+    <hyperlink ref="D6" r:id="rId3" xr:uid="{C20B532B-CF38-45ED-A9A6-B0314F17708B}"/>
+    <hyperlink ref="D8" r:id="rId4" xr:uid="{6C0887D4-947C-4463-A546-6AB836B0B3D8}"/>
+    <hyperlink ref="D9" r:id="rId5" xr:uid="{F0533DB3-A661-4182-888A-949669537D09}"/>
+    <hyperlink ref="D10" r:id="rId6" xr:uid="{3C31B3A0-29AB-41BE-B877-46BE0AC5D6D5}"/>
+    <hyperlink ref="D11" r:id="rId7" xr:uid="{C0DAFC63-62EC-41DB-8DCD-5B75D22A1A2B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3825,13 +3831,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3911,13 +3917,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3928,15 +3934,15 @@
       <c r="C2" s="26"/>
       <c r="D2" s="26"/>
     </row>
-    <row r="3" spans="1:4" ht="42.75">
+    <row r="3" spans="1:4" ht="40.5">
       <c r="A3" s="60" t="s">
         <v>49</v>
       </c>
       <c r="B3" s="156" t="s">
-        <v>307</v>
-      </c>
-      <c r="C3" s="156" t="s">
         <v>308</v>
+      </c>
+      <c r="C3" s="156">
+        <v>2023</v>
       </c>
       <c r="D3" s="192" t="s">
         <v>309</v>
@@ -3947,7 +3953,9 @@
       <c r="B4" s="190" t="s">
         <v>310</v>
       </c>
-      <c r="C4" s="190"/>
+      <c r="C4" s="190">
+        <v>2023</v>
+      </c>
       <c r="D4" s="190"/>
     </row>
     <row r="5" spans="1:4" ht="40.5">
@@ -3989,7 +3997,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>314</v>
@@ -3998,10 +4006,10 @@
         <v>315</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="35.25" customHeight="1">
@@ -4330,13 +4338,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -4383,13 +4391,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -4509,13 +4517,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -5349,7 +5357,7 @@
     </row>
     <row r="41" spans="1:14" ht="16.5">
       <c r="A41" s="79" t="s">
-        <v>79</v>
+        <v>125</v>
       </c>
       <c r="I41" t="s">
         <v>8</v>
@@ -5357,7 +5365,7 @@
     </row>
     <row r="42" spans="1:14" ht="16.5">
       <c r="A42" s="79" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B42" t="s">
         <v>115</v>
@@ -5458,7 +5466,7 @@
         <v>97</v>
       </c>
       <c r="D52" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="16.5">
@@ -5493,13 +5501,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -5515,13 +5523,13 @@
         <v>7</v>
       </c>
       <c r="B3" s="100" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C3" s="100" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D3" s="100" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="40.5" customHeight="1">
@@ -5529,13 +5537,13 @@
         <v>12</v>
       </c>
       <c r="B4" s="101" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C4" s="101" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D4" s="149" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16.5">
@@ -5543,7 +5551,7 @@
         <v>13</v>
       </c>
       <c r="B5" s="102" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C5" s="102"/>
       <c r="D5" s="102"/>
@@ -5561,13 +5569,13 @@
         <v>15</v>
       </c>
       <c r="B7" s="103" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C7" s="103">
         <v>2022</v>
       </c>
       <c r="D7" s="150" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16.5">
@@ -5575,13 +5583,13 @@
         <v>18</v>
       </c>
       <c r="B8" s="104" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C8" s="104">
         <v>2022</v>
       </c>
       <c r="D8" s="151" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="16.5">
@@ -5589,13 +5597,13 @@
         <v>28</v>
       </c>
       <c r="B9" s="104" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C9" s="104">
         <v>2022</v>
       </c>
       <c r="D9" s="151" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -5611,13 +5619,13 @@
         <v>35</v>
       </c>
       <c r="B11" s="105" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C11" s="105" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D11" s="152" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="16.5">
@@ -5625,13 +5633,13 @@
         <v>37</v>
       </c>
       <c r="B12" s="106" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C12" s="106" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D12" s="153" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="16.5">
@@ -5639,13 +5647,13 @@
         <v>38</v>
       </c>
       <c r="B13" s="106" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C13" s="106" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D13" s="153" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="49.5" customHeight="1">
@@ -5653,13 +5661,13 @@
         <v>43</v>
       </c>
       <c r="B14" s="154" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C14" s="106" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D14" s="153" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -5675,13 +5683,13 @@
         <v>49</v>
       </c>
       <c r="B16" s="156" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C16" s="107">
         <v>2024</v>
       </c>
       <c r="D16" s="155" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -5697,13 +5705,13 @@
         <v>66</v>
       </c>
       <c r="B18" s="108" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C18" s="108" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D18" s="108" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="33.75" customHeight="1">
@@ -5711,13 +5719,13 @@
         <v>69</v>
       </c>
       <c r="B19" s="157" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C19" s="157" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D19" s="157" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="34.5" customHeight="1">
@@ -5725,27 +5733,27 @@
         <v>71</v>
       </c>
       <c r="B20" s="158" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C20" s="110" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D20" s="159" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="28.5">
       <c r="A21" s="79" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B21" s="160" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C21" s="111">
         <v>2022</v>
       </c>
       <c r="D21" s="161" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -5761,18 +5769,18 @@
         <v>88</v>
       </c>
       <c r="B23" s="123" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C23" s="123" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D23" s="123" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="51.75" customHeight="1">
       <c r="D24" s="162" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -5809,13 +5817,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -5831,19 +5839,19 @@
         <v>15</v>
       </c>
       <c r="B3" s="163" t="s">
-        <v>165</v>
-      </c>
-      <c r="C3" s="50">
-        <v>2022</v>
+        <v>166</v>
+      </c>
+      <c r="C3" s="200" t="s">
+        <v>167</v>
       </c>
       <c r="D3" s="170" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E3" s="169" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F3" s="169" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="63.75" customHeight="1">
@@ -5851,14 +5859,14 @@
         <v>18</v>
       </c>
       <c r="B4" s="146" t="s">
-        <v>169</v>
-      </c>
-      <c r="C4" s="37">
-        <v>2022</v>
+        <v>171</v>
+      </c>
+      <c r="C4" s="201" t="s">
+        <v>167</v>
       </c>
       <c r="D4" s="37"/>
       <c r="E4" s="169" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="54" customHeight="1">
@@ -5866,14 +5874,14 @@
         <v>20</v>
       </c>
       <c r="B5" s="147" t="s">
-        <v>171</v>
-      </c>
-      <c r="C5" s="37">
-        <v>2022</v>
+        <v>173</v>
+      </c>
+      <c r="C5" s="201" t="s">
+        <v>167</v>
       </c>
       <c r="D5" s="37"/>
       <c r="E5" s="193" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="28.5">
@@ -5881,14 +5889,14 @@
         <v>23</v>
       </c>
       <c r="B6" s="147" t="s">
-        <v>172</v>
-      </c>
-      <c r="C6" s="37">
-        <v>2022</v>
+        <v>174</v>
+      </c>
+      <c r="C6" s="201" t="s">
+        <v>167</v>
       </c>
       <c r="D6" s="37"/>
       <c r="E6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="33" customHeight="1">
@@ -5896,25 +5904,25 @@
         <v>26</v>
       </c>
       <c r="B7" s="147" t="s">
-        <v>174</v>
-      </c>
-      <c r="C7" s="37">
-        <v>2022</v>
+        <v>176</v>
+      </c>
+      <c r="C7" s="201" t="s">
+        <v>167</v>
       </c>
       <c r="D7" s="37"/>
       <c r="E7" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="28.5">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="42.75">
       <c r="A8" s="51" t="s">
         <v>28</v>
       </c>
       <c r="B8" s="147" t="s">
-        <v>176</v>
-      </c>
-      <c r="C8" s="37" t="s">
-        <v>177</v>
+        <v>178</v>
+      </c>
+      <c r="C8" s="201" t="s">
+        <v>179</v>
       </c>
       <c r="D8" s="37"/>
     </row>
@@ -5926,15 +5934,15 @@
       <c r="C9" s="22"/>
       <c r="D9" s="22"/>
     </row>
-    <row r="10" spans="1:6" ht="28.5">
+    <row r="10" spans="1:6" ht="42.75">
       <c r="A10" s="55" t="s">
         <v>43</v>
       </c>
       <c r="B10" s="164" t="s">
-        <v>178</v>
-      </c>
-      <c r="C10" s="56" t="s">
-        <v>177</v>
+        <v>180</v>
+      </c>
+      <c r="C10" s="202" t="s">
+        <v>179</v>
       </c>
       <c r="D10" s="56"/>
     </row>
@@ -5951,10 +5959,10 @@
         <v>66</v>
       </c>
       <c r="B12" s="165" t="s">
+        <v>181</v>
+      </c>
+      <c r="C12" s="203" t="s">
         <v>179</v>
-      </c>
-      <c r="C12" s="77" t="s">
-        <v>177</v>
       </c>
       <c r="D12" s="77"/>
     </row>
@@ -5963,41 +5971,39 @@
         <v>69</v>
       </c>
       <c r="B13" s="166" t="s">
-        <v>180</v>
-      </c>
-      <c r="C13" s="45" t="s">
-        <v>177</v>
+        <v>182</v>
+      </c>
+      <c r="C13" s="204" t="s">
+        <v>179</v>
       </c>
       <c r="D13" s="45"/>
     </row>
-    <row r="14" spans="1:6" ht="16.5">
+    <row r="14" spans="1:6" ht="42.75">
       <c r="A14" s="79" t="s">
         <v>76</v>
       </c>
       <c r="B14" s="168" t="s">
-        <v>181</v>
-      </c>
-      <c r="C14" s="80" t="s">
-        <v>177</v>
+        <v>183</v>
+      </c>
+      <c r="C14" s="205" t="s">
+        <v>179</v>
       </c>
       <c r="D14" s="80"/>
     </row>
-    <row r="15" spans="1:6" ht="28.5">
+    <row r="15" spans="1:6" ht="42.75">
       <c r="A15" s="79" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B15" s="167" t="s">
-        <v>183</v>
-      </c>
-      <c r="C15" s="81" t="s">
-        <v>177</v>
+        <v>185</v>
+      </c>
+      <c r="C15" s="206" t="s">
+        <v>179</v>
       </c>
       <c r="D15" s="81"/>
     </row>
     <row r="16" spans="1:6" ht="147.75" customHeight="1">
-      <c r="C16" s="169" t="s">
-        <v>184</v>
-      </c>
+      <c r="C16" s="169"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6024,13 +6030,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -6047,14 +6053,14 @@
         <v>15</v>
       </c>
       <c r="B3" s="103" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C3" s="103"/>
       <c r="D3" s="172" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E3" s="162" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5">
@@ -6062,7 +6068,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="104" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C4" s="104"/>
       <c r="D4" s="104"/>
@@ -6072,10 +6078,10 @@
         <v>20</v>
       </c>
       <c r="B5" s="171" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C5" s="171" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D5" s="104"/>
     </row>
@@ -6084,10 +6090,10 @@
         <v>23</v>
       </c>
       <c r="B6" s="104" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C6" s="171" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D6" s="104"/>
     </row>
@@ -6096,60 +6102,60 @@
         <v>28</v>
       </c>
       <c r="B7" s="171" t="s">
+        <v>193</v>
+      </c>
+      <c r="C7" s="171" t="s">
         <v>192</v>
-      </c>
-      <c r="C7" s="171" t="s">
-        <v>191</v>
       </c>
       <c r="D7" s="104"/>
     </row>
     <row r="8" spans="1:5" ht="28.5">
       <c r="A8" s="175"/>
       <c r="B8" s="176" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C8" s="176" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D8" s="177"/>
     </row>
     <row r="9" spans="1:5" ht="37.5" customHeight="1">
       <c r="A9" s="175"/>
       <c r="B9" s="176" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C9" s="176" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D9" s="177"/>
     </row>
     <row r="10" spans="1:5" ht="39.75" customHeight="1">
       <c r="A10" s="175"/>
       <c r="B10" s="176" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C10" s="176" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D10" s="177"/>
     </row>
     <row r="11" spans="1:5" ht="28.5">
       <c r="A11" s="175"/>
       <c r="B11" s="176" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C11" s="176" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D11" s="177"/>
     </row>
     <row r="12" spans="1:5" ht="37.5" customHeight="1">
       <c r="A12" s="175"/>
       <c r="B12" s="176" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C12" s="176" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D12" s="177"/>
     </row>
@@ -6158,20 +6164,20 @@
         <v>31</v>
       </c>
       <c r="B13" s="176" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C13" s="176" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D13" s="177"/>
     </row>
     <row r="14" spans="1:5" ht="28.5">
       <c r="A14" s="12"/>
       <c r="B14" s="173" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C14" s="173" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D14" s="113"/>
     </row>
@@ -6188,10 +6194,10 @@
         <v>58</v>
       </c>
       <c r="B16" s="70" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C16" s="114" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D16" s="114"/>
     </row>
@@ -6200,10 +6206,10 @@
         <v>60</v>
       </c>
       <c r="B17" s="114" t="s">
+        <v>208</v>
+      </c>
+      <c r="C17" s="114" t="s">
         <v>207</v>
-      </c>
-      <c r="C17" s="114" t="s">
-        <v>206</v>
       </c>
       <c r="D17" s="114"/>
     </row>
@@ -6220,7 +6226,7 @@
         <v>66</v>
       </c>
       <c r="B19" s="174" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C19" s="108">
         <v>6</v>
@@ -6232,7 +6238,7 @@
         <v>69</v>
       </c>
       <c r="B20" s="157" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C20" s="109">
         <v>6</v>
@@ -6241,70 +6247,70 @@
     </row>
     <row r="21" spans="1:5" ht="28.5">
       <c r="A21" s="79" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B21" s="160" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C21" s="160" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D21" s="111"/>
     </row>
     <row r="22" spans="1:5" ht="44.25" customHeight="1">
       <c r="A22" s="79"/>
       <c r="B22" s="160" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C22" s="160" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D22" s="111"/>
     </row>
     <row r="23" spans="1:5" ht="38.25" customHeight="1">
       <c r="A23" s="79"/>
       <c r="B23" s="160" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C23" s="160" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D23" s="111"/>
     </row>
     <row r="24" spans="1:5" ht="39.75" customHeight="1">
       <c r="A24" s="79"/>
       <c r="B24" s="160" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C24" s="160" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D24" s="111"/>
     </row>
     <row r="25" spans="1:5" ht="36" customHeight="1">
       <c r="A25" s="79"/>
       <c r="B25" s="160" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C25" s="160" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D25" s="111"/>
     </row>
     <row r="26" spans="1:5" ht="36.75" customHeight="1">
       <c r="A26" s="79"/>
       <c r="B26" s="160" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C26" s="160" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D26" s="111"/>
     </row>
     <row r="27" spans="1:5" ht="16.5">
       <c r="A27" s="79"/>
       <c r="B27" s="160" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C27" s="160">
         <v>6</v>
@@ -6314,7 +6320,7 @@
     <row r="28" spans="1:5" ht="16.5">
       <c r="A28" s="79"/>
       <c r="B28" s="160" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C28" s="160">
         <v>6</v>
@@ -6324,7 +6330,7 @@
     <row r="29" spans="1:5" ht="16.5">
       <c r="A29" s="79"/>
       <c r="B29" s="111" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C29" s="111">
         <v>6</v>
@@ -6344,33 +6350,33 @@
         <v>88</v>
       </c>
       <c r="B31" s="148" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C31" s="148" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D31" s="85"/>
     </row>
     <row r="32" spans="1:5" ht="53.25">
       <c r="A32" s="85"/>
       <c r="B32" s="148" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C32" s="148" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D32" s="85"/>
       <c r="E32" s="162" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="28.5">
       <c r="A33" s="85"/>
       <c r="B33" s="148" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C33" s="148" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D33" s="85"/>
       <c r="E33" s="162"/>
@@ -6378,10 +6384,10 @@
     <row r="34" spans="1:5" ht="28.5">
       <c r="A34" s="85"/>
       <c r="B34" s="148" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C34" s="148" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D34" s="85"/>
       <c r="E34" s="162"/>
@@ -6389,7 +6395,7 @@
     <row r="35" spans="1:5" ht="28.5">
       <c r="A35" s="85"/>
       <c r="B35" s="148" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C35" s="148">
         <v>6</v>
@@ -6400,10 +6406,10 @@
     <row r="36" spans="1:5" ht="28.5">
       <c r="A36" s="85"/>
       <c r="B36" s="148" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D36" s="85"/>
       <c r="E36" s="162"/>
@@ -6421,10 +6427,10 @@
         <v>92</v>
       </c>
       <c r="B38" s="178" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C38" s="178" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D38" s="115"/>
     </row>
@@ -6433,10 +6439,10 @@
         <v>93</v>
       </c>
       <c r="B39" s="179" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C39" s="179" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D39" s="116"/>
     </row>
@@ -6445,10 +6451,10 @@
         <v>94</v>
       </c>
       <c r="B40" s="179" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C40" s="179" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D40" s="116"/>
     </row>
@@ -6457,14 +6463,14 @@
         <v>95</v>
       </c>
       <c r="B41" s="144" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C41" s="116" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D41" s="116"/>
       <c r="E41" s="162" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="80.25">
@@ -6472,14 +6478,14 @@
         <v>97</v>
       </c>
       <c r="B42" s="116" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C42" s="116" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D42" s="116"/>
       <c r="E42" s="162" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="28.5">
@@ -6487,10 +6493,10 @@
         <v>98</v>
       </c>
       <c r="B43" s="183" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C43" s="183" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D43" s="182"/>
       <c r="E43" s="162"/>
@@ -6498,16 +6504,16 @@
     <row r="44" spans="1:5" ht="28.5">
       <c r="A44" s="95"/>
       <c r="B44" s="180" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C44" s="180" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D44" s="117"/>
     </row>
     <row r="45" spans="1:5" ht="126" customHeight="1">
       <c r="C45" s="162" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -6532,13 +6538,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -6554,7 +6560,7 @@
         <v>15</v>
       </c>
       <c r="B3" s="132" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C3" s="103">
         <v>2023</v>
@@ -6566,7 +6572,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="132" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C4" s="104">
         <v>2023</v>
@@ -6576,7 +6582,7 @@
     <row r="5" spans="1:4" ht="16.5">
       <c r="A5" s="51"/>
       <c r="B5" s="133" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C5" s="104">
         <v>2023</v>
@@ -6588,7 +6594,7 @@
         <v>28</v>
       </c>
       <c r="B6" s="133" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C6" s="104">
         <v>2023</v>
@@ -6608,7 +6614,7 @@
         <v>43</v>
       </c>
       <c r="B8" s="135" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C8" s="106">
         <v>2023</v>
@@ -6628,7 +6634,7 @@
         <v>58</v>
       </c>
       <c r="B10" s="137" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C10" s="114">
         <v>2023</v>
@@ -6640,7 +6646,7 @@
         <v>60</v>
       </c>
       <c r="B11" s="137" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C11" s="114">
         <v>2023</v>
@@ -6660,7 +6666,7 @@
         <v>76</v>
       </c>
       <c r="B13" s="139" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C13" s="110">
         <v>2023</v>
@@ -6669,10 +6675,10 @@
     </row>
     <row r="14" spans="1:4" ht="16.5">
       <c r="A14" s="79" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B14" s="139" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C14" s="111">
         <v>2023</v>
@@ -6692,7 +6698,7 @@
         <v>88</v>
       </c>
       <c r="B16" s="141" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C16" s="112">
         <v>2023</v>
@@ -6702,7 +6708,7 @@
     <row r="17" spans="1:4" ht="57">
       <c r="A17" s="85"/>
       <c r="B17" s="142" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C17" s="112">
         <v>2023</v>
@@ -6712,7 +6718,7 @@
     <row r="18" spans="1:4" ht="16.5">
       <c r="A18" s="85"/>
       <c r="B18" s="142" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C18" s="112">
         <v>2023</v>
@@ -6722,7 +6728,7 @@
     <row r="19" spans="1:4" ht="28.5">
       <c r="A19" s="85"/>
       <c r="B19" s="142" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C19" s="112">
         <v>2023</v>
@@ -6742,7 +6748,7 @@
         <v>95</v>
       </c>
       <c r="B21" s="144" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C21" s="116">
         <v>2023</v>
@@ -6752,7 +6758,7 @@
     <row r="22" spans="1:4" ht="42.75">
       <c r="A22" s="90"/>
       <c r="B22" s="145" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C22" s="90">
         <v>2023</v>
@@ -6778,13 +6784,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -6800,22 +6806,22 @@
         <v>15</v>
       </c>
       <c r="B3" s="184" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C3" s="103">
         <v>2023</v>
       </c>
       <c r="D3" s="172" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E3" s="169" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.5" customHeight="1">
       <c r="A4" s="185"/>
       <c r="B4" s="186" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C4" s="187">
         <v>2023</v>
@@ -6826,7 +6832,7 @@
     <row r="5" spans="1:5" ht="31.5" customHeight="1">
       <c r="A5" s="185"/>
       <c r="B5" s="186" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C5" s="187">
         <v>2023</v>
@@ -6837,7 +6843,7 @@
     <row r="6" spans="1:5" ht="31.5" customHeight="1">
       <c r="A6" s="185"/>
       <c r="B6" s="186" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C6" s="187">
         <v>2023</v>
@@ -6848,7 +6854,7 @@
     <row r="7" spans="1:5" ht="61.5" customHeight="1">
       <c r="A7" s="185"/>
       <c r="B7" s="186" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C7" s="187">
         <v>2023</v>
@@ -6859,7 +6865,7 @@
     <row r="8" spans="1:5" ht="21.75" customHeight="1">
       <c r="A8" s="185"/>
       <c r="B8" s="186" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C8" s="187">
         <v>2023</v>
@@ -6870,7 +6876,7 @@
     <row r="9" spans="1:5" ht="21.75" customHeight="1">
       <c r="A9" s="185"/>
       <c r="B9" s="186" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C9" s="187">
         <v>2023</v>
@@ -6883,7 +6889,7 @@
         <v>18</v>
       </c>
       <c r="B10" s="171" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C10" s="104">
         <v>2023</v>
@@ -6893,7 +6899,7 @@
     <row r="11" spans="1:5" ht="16.5">
       <c r="A11" s="51"/>
       <c r="B11" s="104" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C11" s="104">
         <v>2023</v>
@@ -6903,7 +6909,7 @@
     <row r="12" spans="1:5" ht="16.5">
       <c r="A12" s="51"/>
       <c r="B12" s="104" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C12" s="104">
         <v>2023</v>
@@ -6913,7 +6919,7 @@
     <row r="13" spans="1:5" ht="42.75">
       <c r="A13" s="51"/>
       <c r="B13" s="171" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C13" s="104">
         <v>2023</v>
@@ -6923,7 +6929,7 @@
     <row r="14" spans="1:5" ht="16.5">
       <c r="A14" s="51"/>
       <c r="B14" s="171" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C14" s="104">
         <v>2023</v>
@@ -6933,7 +6939,7 @@
     <row r="15" spans="1:5" ht="16.5">
       <c r="A15" s="51"/>
       <c r="B15" s="171" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C15" s="104">
         <v>2023</v>
@@ -6943,7 +6949,7 @@
     <row r="16" spans="1:5" ht="57">
       <c r="A16" s="51"/>
       <c r="B16" s="171" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C16" s="104">
         <v>2023</v>
@@ -6953,7 +6959,7 @@
     <row r="17" spans="1:4" ht="16.5">
       <c r="A17" s="51"/>
       <c r="B17" s="171" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C17" s="104">
         <v>2023</v>
@@ -6963,7 +6969,7 @@
     <row r="18" spans="1:4" ht="71.25">
       <c r="A18" s="51"/>
       <c r="B18" s="171" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C18" s="104">
         <v>2023</v>
@@ -6973,7 +6979,7 @@
     <row r="19" spans="1:4" ht="16.5">
       <c r="A19" s="51"/>
       <c r="B19" s="171" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C19" s="104">
         <v>2023</v>
@@ -6983,7 +6989,7 @@
     <row r="20" spans="1:4" ht="57">
       <c r="A20" s="51"/>
       <c r="B20" s="171" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C20" s="104">
         <v>2023</v>
@@ -6993,7 +6999,7 @@
     <row r="21" spans="1:4" ht="16.5">
       <c r="A21" s="51"/>
       <c r="B21" s="171" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C21" s="104">
         <v>2023</v>
@@ -7003,7 +7009,7 @@
     <row r="22" spans="1:4" ht="28.5">
       <c r="A22" s="51"/>
       <c r="B22" s="171" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C22" s="104">
         <v>2023</v>
@@ -7013,7 +7019,7 @@
     <row r="23" spans="1:4" ht="57">
       <c r="A23" s="51"/>
       <c r="B23" s="171" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C23" s="104">
         <v>2023</v>
@@ -7025,7 +7031,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="171" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C24" s="104">
         <v>2023</v>
@@ -7035,7 +7041,7 @@
     <row r="25" spans="1:4" ht="16.5">
       <c r="A25" s="51"/>
       <c r="B25" s="104" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C25" s="104">
         <v>2023</v>
@@ -7047,7 +7053,7 @@
         <v>28</v>
       </c>
       <c r="B26" s="104" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C26" s="104">
         <v>2023</v>
@@ -7057,7 +7063,7 @@
     <row r="27" spans="1:4" ht="16.5">
       <c r="A27" s="51"/>
       <c r="B27" s="104" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C27" s="104">
         <v>2023</v>
@@ -7077,7 +7083,7 @@
         <v>43</v>
       </c>
       <c r="B29" s="154" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C29" s="106">
         <v>2023</v>
@@ -7087,7 +7093,7 @@
     <row r="30" spans="1:4" ht="16.5">
       <c r="A30" s="55"/>
       <c r="B30" s="154" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C30" s="106">
         <v>2023</v>
@@ -7097,7 +7103,7 @@
     <row r="31" spans="1:4" ht="28.5">
       <c r="A31" s="55"/>
       <c r="B31" s="154" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C31" s="106">
         <v>2023</v>
@@ -7107,7 +7113,7 @@
     <row r="32" spans="1:4" ht="16.5">
       <c r="A32" s="55"/>
       <c r="B32" s="154" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C32" s="106">
         <v>2023</v>
@@ -7117,7 +7123,7 @@
     <row r="33" spans="1:4" ht="16.5">
       <c r="A33" s="55"/>
       <c r="B33" s="154" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C33" s="106">
         <v>2023</v>
@@ -7127,7 +7133,7 @@
     <row r="34" spans="1:4" ht="28.5">
       <c r="A34" s="55"/>
       <c r="B34" s="154" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C34" s="106">
         <v>2023</v>
@@ -7137,7 +7143,7 @@
     <row r="35" spans="1:4" ht="28.5">
       <c r="A35" s="55"/>
       <c r="B35" s="154" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C35" s="106">
         <v>2023</v>
@@ -7147,7 +7153,7 @@
     <row r="36" spans="1:4" ht="28.5">
       <c r="A36" s="55"/>
       <c r="B36" s="154" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C36" s="106">
         <v>2023</v>
@@ -7157,7 +7163,7 @@
     <row r="37" spans="1:4" ht="28.5">
       <c r="A37" s="55"/>
       <c r="B37" s="154" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C37" s="106">
         <v>2023</v>
@@ -7167,7 +7173,7 @@
     <row r="38" spans="1:4" ht="28.5">
       <c r="A38" s="55"/>
       <c r="B38" s="154" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C38" s="106">
         <v>2023</v>
@@ -7177,7 +7183,7 @@
     <row r="39" spans="1:4" ht="28.5">
       <c r="A39" s="55"/>
       <c r="B39" s="154" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C39" s="106">
         <v>2023</v>
@@ -7197,7 +7203,7 @@
         <v>66</v>
       </c>
       <c r="B41" s="108" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C41" s="108">
         <v>2023</v>
@@ -7209,7 +7215,7 @@
         <v>69</v>
       </c>
       <c r="B42" s="157" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C42" s="109">
         <v>2023</v>
@@ -7218,10 +7224,10 @@
     </row>
     <row r="43" spans="1:4" ht="28.5">
       <c r="A43" s="79" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B43" s="160" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C43" s="111">
         <v>2023</v>
@@ -7231,7 +7237,7 @@
     <row r="44" spans="1:4" ht="28.5">
       <c r="A44" s="79"/>
       <c r="B44" s="160" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C44" s="111">
         <v>2023</v>
@@ -7251,7 +7257,7 @@
         <v>88</v>
       </c>
       <c r="B46" s="112" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C46" s="112">
         <v>2023</v>
@@ -7261,7 +7267,7 @@
     <row r="47" spans="1:4" ht="16.5">
       <c r="A47" s="85"/>
       <c r="B47" s="112" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C47" s="112">
         <v>2023</v>
@@ -7270,7 +7276,7 @@
     </row>
     <row r="48" spans="1:4" ht="147">
       <c r="C48" s="162" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -7296,13 +7302,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -7318,13 +7324,13 @@
         <v>86</v>
       </c>
       <c r="B3" s="127" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C3" s="112">
         <v>2023</v>
       </c>
       <c r="D3" s="129" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
   </sheetData>
@@ -7349,13 +7355,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -7371,7 +7377,7 @@
         <v>39</v>
       </c>
       <c r="B3" s="106" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C3" s="106"/>
       <c r="D3" s="106"/>
@@ -7398,12 +7404,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MediaServiceKeyPoints xmlns="99eecc7c-9af8-4a20-9690-8dd5901fd572" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7597,15 +7602,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MediaServiceKeyPoints xmlns="99eecc7c-9af8-4a20-9690-8dd5901fd572" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53BF39ED-8412-4A1A-B8D1-D3BEBCC138C5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D765DD3-C5A9-4E60-8819-7516E8229505}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7613,5 +7619,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D765DD3-C5A9-4E60-8819-7516E8229505}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53BF39ED-8412-4A1A-B8D1-D3BEBCC138C5}"/>
 </file>
</xml_diff>